<commit_message>
Updated Description and Outcome Message as requested; added TSGRPID as Output Variable; value_is_literal condition added to Check.
</commit_message>
<xml_diff>
--- a/rules/CORE-000473/negative/01/data/unit-test-coreid-CG0272-negative 1.xlsx
+++ b/rules/CORE-000473/negative/01/data/unit-test-coreid-CG0272-negative 1.xlsx
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -585,9 +585,29 @@
         <v>Patients with Probable Mild to Moderate Alzheimers Disease</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>ts.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>6</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>TSGRPID</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -781,7 +801,7 @@
       <c r="C6" s="4">
         <v>1</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="7">
         <v>1</v>
       </c>
       <c r="E6" s="7" t="str">

</xml_diff>